<commit_message>
Update Excel file with cities for each Egyptian governate
</commit_message>
<xml_diff>
--- a/Egyptian_Governates.xlsx
+++ b/Egyptian_Governates.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Egyptian Governates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Egyptian Governates &amp; Cities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,9 +28,17 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,8 +51,14 @@
         <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,17 +66,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,10 +452,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,6 +465,11 @@
           <t>Governate</t>
         </is>
       </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cities</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -448,6 +477,11 @@
           <t>Alexandria</t>
         </is>
       </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Alexandria, Borg El Arab, Montaza, Sidi Bishr</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -455,6 +489,11 @@
           <t>Aswan</t>
         </is>
       </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Aswan, Abu Simbel, Kom Ombo, Edfu, Daraw</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -462,6 +501,11 @@
           <t>Asyut</t>
         </is>
       </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Asyut, Manfalut, Dayrut, Abydos, Sohag</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -469,6 +513,11 @@
           <t>Beheira</t>
         </is>
       </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Damanhur, Kafr El Dawwar, Rosetta, Edku, Abu Hummus</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -476,6 +525,11 @@
           <t>Beni Suef</t>
         </is>
       </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Beni Suef, El Fashn, Samasta, Ibshaway, Nasser</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -483,6 +537,11 @@
           <t>Cairo</t>
         </is>
       </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Cairo, Heliopolis, Nasr City, New Cairo, 6th of October City</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -490,6 +549,11 @@
           <t>Dakahlia</t>
         </is>
       </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Mansoura, Talkha, Aga, Mit Ghamr, Sherbin</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -497,6 +561,11 @@
           <t>Damietta</t>
         </is>
       </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Damietta, New Damietta, Port Fuad, Kafr El Sheikh</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -504,6 +573,11 @@
           <t>Faiyum</t>
         </is>
       </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Faiyum, Siwa, Karanis, Ibshaway, Sinnuris</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -511,6 +585,11 @@
           <t>Gharbia</t>
         </is>
       </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Tanta, Kafr El Zayat, Samannud, Zifta, Mahalla</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -518,6 +597,11 @@
           <t>Giza</t>
         </is>
       </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Giza, 6th of October, Helwan, Badrasheen, Dahshur</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -525,6 +609,11 @@
           <t>Helwan</t>
         </is>
       </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Helwan, Maadi, Wadi Hof, Ain Sukhna, Tura</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -532,6 +621,11 @@
           <t>Ismailia</t>
         </is>
       </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Ismailia, Port Said, Suez, El Qantara, Fayid</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -539,6 +633,11 @@
           <t>Kafr El Sheikh</t>
         </is>
       </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Kafr El Sheikh, Dessouk, Balamun, El Riyad, Sidi Salem</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -546,6 +645,11 @@
           <t>Kalyubia</t>
         </is>
       </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Benha, Qalyub, Shubra El Khaimah, Helwan, 10th of Ramadan</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -553,6 +657,11 @@
           <t>Luxor</t>
         </is>
       </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Luxor, Karnak, Thebes, West Bank, Valley of the Kings</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -560,6 +669,11 @@
           <t>Matruh</t>
         </is>
       </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Matruh, Siwa, Salloum, Sidi Barrani, Alamein</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -567,6 +681,11 @@
           <t>Minya</t>
         </is>
       </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Minya, Samalut, Beni Hassan, Hermopolis, El Minya</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -574,6 +693,11 @@
           <t>Monufia</t>
         </is>
       </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Shebin El Kom, Menouf, Shibin El Qanater, Sadat City, Bagour</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -581,6 +705,11 @@
           <t>New Valley</t>
         </is>
       </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Kharga, Dakhla, Mut, Balat, Farafra</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -588,6 +717,11 @@
           <t>North Sinai</t>
         </is>
       </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Arish, Rafah, Sheikh Zuwaid, Bir El Abd, El Qantara</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -595,6 +729,11 @@
           <t>Port Said</t>
         </is>
       </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Port Said, Port Fuad, El Gamil, El Zohour, PORT SAID</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -602,6 +741,11 @@
           <t>Qena</t>
         </is>
       </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Qena, Nag Hammadi, Dendera, Abydos, Coptos</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -609,6 +753,11 @@
           <t>Red Sea</t>
         </is>
       </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Hurghada, Safaga, Quseir, Marsa Alam, Shalateen</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -616,6 +765,11 @@
           <t>Sharqia</t>
         </is>
       </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Zagazig, Ismailia, Belbeis, 10th of Ramadan, Maadi</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -623,11 +777,21 @@
           <t>South Sinai</t>
         </is>
       </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Sharm El Sheikh, Dahab, Nuweiba, Saint Catherine, Taba</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Suez</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Suez, Ain Sukhna, Ataqa, El Ganayen, Fayid</t>
         </is>
       </c>
     </row>

</xml_diff>